<commit_message>
ejercicio 62 con video
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/matricula_asistencia_notas_Caucasia_2026-2.xlsx
+++ b/9_asistencia_evaluacion/matricula_asistencia_notas_Caucasia_2026-2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B794A4C-689C-4D43-86EC-C140409F423E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976D838E-FADD-465B-908A-D4B3EF9CCB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="107">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -356,6 +356,9 @@
   </si>
   <si>
     <t>Walter Antonio Perez Guzman</t>
+  </si>
+  <si>
+    <t>perezguzmanwalterantonio14@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -798,7 +801,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -925,6 +928,99 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="16" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -955,15 +1051,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1009,87 +1096,6 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1190,10 +1196,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="16" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1689,28 +1691,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="102"/>
+      <c r="B1" s="102"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="103"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="99" t="s">
+      <c r="A2" s="100" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="99"/>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99"/>
-      <c r="H2" s="99"/>
+      <c r="B2" s="100"/>
+      <c r="C2" s="100"/>
+      <c r="D2" s="100"/>
+      <c r="E2" s="100"/>
+      <c r="F2" s="100"/>
+      <c r="G2" s="100"/>
+      <c r="H2" s="100"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -2096,7 +2098,7 @@
         <v>1033261244</v>
       </c>
       <c r="E20" s="14"/>
-      <c r="F20" s="133">
+      <c r="F20">
         <v>3215036126</v>
       </c>
       <c r="G20" s="43" t="s">
@@ -2162,7 +2164,7 @@
         <v>1038116237</v>
       </c>
       <c r="E23" s="14"/>
-      <c r="F23" s="133">
+      <c r="F23">
         <v>3147879724</v>
       </c>
       <c r="G23" s="43" t="s">
@@ -2507,11 +2509,19 @@
       <c r="B39" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
+      <c r="C39" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="D39" s="15">
+        <v>1040502849</v>
+      </c>
       <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="17"/>
+      <c r="F39" s="14">
+        <v>3218908879</v>
+      </c>
+      <c r="G39" s="17" t="s">
+        <v>106</v>
+      </c>
       <c r="H39" s="14"/>
     </row>
     <row r="40" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
@@ -2845,172 +2855,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="110" t="s">
+      <c r="B1" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="110"/>
-      <c r="D1" s="110"/>
-      <c r="E1" s="110"/>
-      <c r="F1" s="110"/>
-      <c r="G1" s="110"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="110"/>
-      <c r="K1" s="110"/>
-      <c r="L1" s="110"/>
-      <c r="M1" s="110"/>
-      <c r="N1" s="110"/>
-      <c r="O1" s="110"/>
-      <c r="P1" s="110"/>
-      <c r="Q1" s="110"/>
-      <c r="R1" s="110"/>
-      <c r="S1" s="110"/>
-      <c r="T1" s="110"/>
-      <c r="U1" s="110"/>
-      <c r="V1" s="110"/>
-      <c r="W1" s="110"/>
-      <c r="X1" s="110"/>
-      <c r="Y1" s="110"/>
-      <c r="Z1" s="110"/>
-      <c r="AA1" s="110"/>
-      <c r="AB1" s="110"/>
-      <c r="AC1" s="110"/>
-      <c r="AD1" s="110"/>
-      <c r="AE1" s="110"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
+      <c r="P1" s="111"/>
+      <c r="Q1" s="111"/>
+      <c r="R1" s="111"/>
+      <c r="S1" s="111"/>
+      <c r="T1" s="111"/>
+      <c r="U1" s="111"/>
+      <c r="V1" s="111"/>
+      <c r="W1" s="111"/>
+      <c r="X1" s="111"/>
+      <c r="Y1" s="111"/>
+      <c r="Z1" s="111"/>
+      <c r="AA1" s="111"/>
+      <c r="AB1" s="111"/>
+      <c r="AC1" s="111"/>
+      <c r="AD1" s="111"/>
+      <c r="AE1" s="111"/>
     </row>
     <row r="2" spans="1:31" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="97" t="s">
+      <c r="A2" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="95" t="s">
+      <c r="B2" s="71" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="97" t="s">
+      <c r="C2" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="126" t="s">
+      <c r="D2" s="127" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="127"/>
-      <c r="F2" s="127"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="111" t="s">
+      <c r="E2" s="128"/>
+      <c r="F2" s="128"/>
+      <c r="G2" s="128"/>
+      <c r="H2" s="129"/>
+      <c r="I2" s="112" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="112"/>
-      <c r="K2" s="112"/>
-      <c r="L2" s="112"/>
-      <c r="M2" s="112"/>
-      <c r="N2" s="112"/>
-      <c r="O2" s="112"/>
-      <c r="P2" s="112"/>
-      <c r="Q2" s="113"/>
-      <c r="R2" s="120" t="s">
+      <c r="J2" s="113"/>
+      <c r="K2" s="113"/>
+      <c r="L2" s="113"/>
+      <c r="M2" s="113"/>
+      <c r="N2" s="113"/>
+      <c r="O2" s="113"/>
+      <c r="P2" s="113"/>
+      <c r="Q2" s="114"/>
+      <c r="R2" s="121" t="s">
         <v>20</v>
       </c>
-      <c r="S2" s="121"/>
-      <c r="T2" s="121"/>
-      <c r="U2" s="121"/>
-      <c r="V2" s="121"/>
-      <c r="W2" s="121"/>
-      <c r="X2" s="121"/>
-      <c r="Y2" s="121"/>
-      <c r="Z2" s="122"/>
-      <c r="AA2" s="103" t="s">
+      <c r="S2" s="122"/>
+      <c r="T2" s="122"/>
+      <c r="U2" s="122"/>
+      <c r="V2" s="122"/>
+      <c r="W2" s="122"/>
+      <c r="X2" s="122"/>
+      <c r="Y2" s="122"/>
+      <c r="Z2" s="123"/>
+      <c r="AA2" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="AB2" s="104"/>
-      <c r="AC2" s="104"/>
-      <c r="AD2" s="104"/>
-      <c r="AE2" s="105"/>
+      <c r="AB2" s="105"/>
+      <c r="AC2" s="105"/>
+      <c r="AD2" s="105"/>
+      <c r="AE2" s="106"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="98"/>
-      <c r="B3" s="96"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="129" t="s">
+      <c r="A3" s="74"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="130" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="130"/>
-      <c r="F3" s="130"/>
-      <c r="G3" s="130"/>
-      <c r="H3" s="131"/>
-      <c r="I3" s="114" t="s">
+      <c r="E3" s="131"/>
+      <c r="F3" s="131"/>
+      <c r="G3" s="131"/>
+      <c r="H3" s="132"/>
+      <c r="I3" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="115"/>
-      <c r="K3" s="115"/>
-      <c r="L3" s="115"/>
-      <c r="M3" s="115"/>
-      <c r="N3" s="115"/>
-      <c r="O3" s="115"/>
-      <c r="P3" s="115"/>
-      <c r="Q3" s="116"/>
-      <c r="R3" s="123" t="s">
+      <c r="J3" s="116"/>
+      <c r="K3" s="116"/>
+      <c r="L3" s="116"/>
+      <c r="M3" s="116"/>
+      <c r="N3" s="116"/>
+      <c r="O3" s="116"/>
+      <c r="P3" s="116"/>
+      <c r="Q3" s="117"/>
+      <c r="R3" s="124" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="124"/>
-      <c r="T3" s="124"/>
-      <c r="U3" s="124"/>
-      <c r="V3" s="124"/>
-      <c r="W3" s="124"/>
-      <c r="X3" s="124"/>
-      <c r="Y3" s="124"/>
-      <c r="Z3" s="125"/>
-      <c r="AA3" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="107"/>
-      <c r="AC3" s="107"/>
-      <c r="AD3" s="107"/>
-      <c r="AE3" s="108"/>
+      <c r="S3" s="125"/>
+      <c r="T3" s="125"/>
+      <c r="U3" s="125"/>
+      <c r="V3" s="125"/>
+      <c r="W3" s="125"/>
+      <c r="X3" s="125"/>
+      <c r="Y3" s="125"/>
+      <c r="Z3" s="126"/>
+      <c r="AA3" s="107" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="108"/>
+      <c r="AC3" s="108"/>
+      <c r="AD3" s="108"/>
+      <c r="AE3" s="109"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="98"/>
-      <c r="B4" s="96"/>
-      <c r="C4" s="98"/>
-      <c r="D4" s="132" t="s">
+      <c r="A4" s="74"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="133" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="118"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="120"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="117" t="s">
+      <c r="I4" s="118" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="118"/>
-      <c r="K4" s="118"/>
-      <c r="L4" s="118"/>
-      <c r="M4" s="118"/>
-      <c r="N4" s="118"/>
-      <c r="O4" s="118"/>
-      <c r="P4" s="119"/>
+      <c r="J4" s="119"/>
+      <c r="K4" s="119"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119"/>
+      <c r="P4" s="120"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="117" t="s">
+      <c r="R4" s="118" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="118"/>
-      <c r="T4" s="118"/>
-      <c r="U4" s="118"/>
-      <c r="V4" s="118"/>
-      <c r="W4" s="118"/>
-      <c r="X4" s="118"/>
-      <c r="Y4" s="119"/>
+      <c r="S4" s="119"/>
+      <c r="T4" s="119"/>
+      <c r="U4" s="119"/>
+      <c r="V4" s="119"/>
+      <c r="W4" s="119"/>
+      <c r="X4" s="119"/>
+      <c r="Y4" s="120"/>
       <c r="Z4" s="12"/>
-      <c r="AA4" s="109" t="s">
+      <c r="AA4" s="110" t="s">
         <v>24</v>
       </c>
-      <c r="AB4" s="109"/>
-      <c r="AC4" s="109"/>
-      <c r="AD4" s="109"/>
+      <c r="AB4" s="110"/>
+      <c r="AC4" s="110"/>
+      <c r="AD4" s="110"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="98"/>
-      <c r="B5" s="96"/>
-      <c r="C5" s="98"/>
+      <c r="A5" s="74"/>
+      <c r="B5" s="72"/>
+      <c r="C5" s="74"/>
       <c r="D5" s="33"/>
       <c r="E5" s="33"/>
       <c r="F5" s="33"/>
@@ -3018,16 +3028,16 @@
       <c r="H5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="134">
+      <c r="I5" s="44">
         <v>46258</v>
       </c>
-      <c r="J5" s="134">
+      <c r="J5" s="44">
         <v>46259</v>
       </c>
-      <c r="K5" s="134">
+      <c r="K5" s="44">
         <v>46260</v>
       </c>
-      <c r="L5" s="134">
+      <c r="L5" s="44">
         <v>46261</v>
       </c>
       <c r="M5" s="28"/>
@@ -4921,7 +4931,7 @@
       </c>
       <c r="C41" s="21">
         <f>+Inscritos!D39</f>
-        <v>0</v>
+        <v>1040502849</v>
       </c>
       <c r="D41" s="13"/>
       <c r="E41" s="13"/>
@@ -6288,123 +6298,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="75"/>
+      <c r="O1" s="75"/>
+      <c r="P1" s="75"/>
+      <c r="Q1" s="75"/>
+      <c r="R1" s="75"/>
+      <c r="S1" s="75"/>
+      <c r="T1" s="75"/>
     </row>
     <row r="2" spans="1:20" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="81" t="s">
+      <c r="A2" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="95" t="s">
+      <c r="B2" s="71" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="97" t="s">
+      <c r="C2" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="72" t="str">
+      <c r="D2" s="45" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="73"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="72" t="str">
+      <c r="E2" s="46"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="45" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="74"/>
-      <c r="L2" s="72" t="s">
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="74"/>
-      <c r="Q2" s="72" t="str">
+      <c r="M2" s="46"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="45" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="73"/>
-      <c r="S2" s="73"/>
-      <c r="T2" s="74"/>
+      <c r="R2" s="46"/>
+      <c r="S2" s="46"/>
+      <c r="T2" s="47"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="82"/>
-      <c r="B3" s="96"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="89" t="s">
+      <c r="A3" s="58"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="90"/>
-      <c r="F3" s="91"/>
-      <c r="G3" s="83" t="s">
+      <c r="E3" s="66"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="84"/>
-      <c r="I3" s="84"/>
-      <c r="J3" s="84"/>
-      <c r="K3" s="85"/>
-      <c r="L3" s="66" t="s">
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="68"/>
-      <c r="Q3" s="75" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="76"/>
-      <c r="S3" s="76"/>
-      <c r="T3" s="77"/>
+      <c r="M3" s="95"/>
+      <c r="N3" s="95"/>
+      <c r="O3" s="95"/>
+      <c r="P3" s="96"/>
+      <c r="Q3" s="48" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="49"/>
+      <c r="S3" s="49"/>
+      <c r="T3" s="50"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="82"/>
-      <c r="B4" s="96"/>
-      <c r="C4" s="98"/>
-      <c r="D4" s="92"/>
-      <c r="E4" s="93"/>
-      <c r="F4" s="94"/>
-      <c r="G4" s="86"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="88"/>
-      <c r="L4" s="69"/>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="71"/>
-      <c r="Q4" s="78"/>
-      <c r="R4" s="79"/>
-      <c r="S4" s="79"/>
-      <c r="T4" s="80"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="97"/>
+      <c r="M4" s="98"/>
+      <c r="N4" s="98"/>
+      <c r="O4" s="98"/>
+      <c r="P4" s="99"/>
+      <c r="Q4" s="51"/>
+      <c r="R4" s="52"/>
+      <c r="S4" s="52"/>
+      <c r="T4" s="53"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="82"/>
-      <c r="B5" s="96"/>
-      <c r="C5" s="98"/>
+      <c r="A5" s="58"/>
+      <c r="B5" s="72"/>
+      <c r="C5" s="74"/>
       <c r="D5" s="22">
         <v>0.75</v>
       </c>
@@ -7945,7 +7955,7 @@
       </c>
       <c r="C41" s="18">
         <f>+Inscritos!D39</f>
-        <v>0</v>
+        <v>1040502849</v>
       </c>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
@@ -8986,195 +8996,186 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D66" s="48" t="s">
+      <c r="D66" s="79" t="s">
         <v>26</v>
       </c>
-      <c r="E66" s="51" t="s">
+      <c r="E66" s="82" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="45" t="s">
+      <c r="G66" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="60" t="s">
+      <c r="H66" s="88" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="60" t="s">
+      <c r="I66" s="88" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="45" t="s">
+      <c r="J66" s="76" t="s">
         <v>11</v>
       </c>
       <c r="L66" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="57" t="s">
+      <c r="M66" s="85" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="57" t="s">
+      <c r="N66" s="85" t="s">
         <v>10</v>
       </c>
       <c r="O66" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="63" t="s">
+      <c r="Q66" s="91" t="s">
         <v>26</v>
       </c>
-      <c r="R66" s="63" t="s">
+      <c r="R66" s="91" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="63" t="s">
+      <c r="S66" s="91" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D67" s="49"/>
-      <c r="E67" s="52"/>
-      <c r="G67" s="46"/>
-      <c r="H67" s="61"/>
-      <c r="I67" s="61"/>
-      <c r="J67" s="46"/>
+      <c r="D67" s="80"/>
+      <c r="E67" s="83"/>
+      <c r="G67" s="77"/>
+      <c r="H67" s="89"/>
+      <c r="I67" s="89"/>
+      <c r="J67" s="77"/>
       <c r="L67" s="55"/>
-      <c r="M67" s="58"/>
-      <c r="N67" s="58"/>
+      <c r="M67" s="86"/>
+      <c r="N67" s="86"/>
       <c r="O67" s="55"/>
-      <c r="Q67" s="64"/>
-      <c r="R67" s="64"/>
-      <c r="S67" s="64"/>
+      <c r="Q67" s="92"/>
+      <c r="R67" s="92"/>
+      <c r="S67" s="92"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D68" s="49"/>
-      <c r="E68" s="52"/>
-      <c r="G68" s="46"/>
-      <c r="H68" s="61"/>
-      <c r="I68" s="61"/>
-      <c r="J68" s="46"/>
+      <c r="D68" s="80"/>
+      <c r="E68" s="83"/>
+      <c r="G68" s="77"/>
+      <c r="H68" s="89"/>
+      <c r="I68" s="89"/>
+      <c r="J68" s="77"/>
       <c r="L68" s="55"/>
-      <c r="M68" s="58"/>
-      <c r="N68" s="58"/>
+      <c r="M68" s="86"/>
+      <c r="N68" s="86"/>
       <c r="O68" s="55"/>
-      <c r="Q68" s="64"/>
-      <c r="R68" s="64"/>
-      <c r="S68" s="64"/>
+      <c r="Q68" s="92"/>
+      <c r="R68" s="92"/>
+      <c r="S68" s="92"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D69" s="49"/>
-      <c r="E69" s="52"/>
-      <c r="G69" s="46"/>
-      <c r="H69" s="61"/>
-      <c r="I69" s="61"/>
-      <c r="J69" s="46"/>
+      <c r="D69" s="80"/>
+      <c r="E69" s="83"/>
+      <c r="G69" s="77"/>
+      <c r="H69" s="89"/>
+      <c r="I69" s="89"/>
+      <c r="J69" s="77"/>
       <c r="L69" s="55"/>
-      <c r="M69" s="58"/>
-      <c r="N69" s="58"/>
+      <c r="M69" s="86"/>
+      <c r="N69" s="86"/>
       <c r="O69" s="55"/>
-      <c r="Q69" s="64"/>
-      <c r="R69" s="64"/>
-      <c r="S69" s="64"/>
+      <c r="Q69" s="92"/>
+      <c r="R69" s="92"/>
+      <c r="S69" s="92"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D70" s="49"/>
-      <c r="E70" s="52"/>
-      <c r="G70" s="46"/>
-      <c r="H70" s="61"/>
-      <c r="I70" s="61"/>
-      <c r="J70" s="46"/>
+      <c r="D70" s="80"/>
+      <c r="E70" s="83"/>
+      <c r="G70" s="77"/>
+      <c r="H70" s="89"/>
+      <c r="I70" s="89"/>
+      <c r="J70" s="77"/>
       <c r="L70" s="55"/>
-      <c r="M70" s="58"/>
-      <c r="N70" s="58"/>
+      <c r="M70" s="86"/>
+      <c r="N70" s="86"/>
       <c r="O70" s="55"/>
-      <c r="Q70" s="64"/>
-      <c r="R70" s="64"/>
-      <c r="S70" s="64"/>
+      <c r="Q70" s="92"/>
+      <c r="R70" s="92"/>
+      <c r="S70" s="92"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D71" s="49"/>
-      <c r="E71" s="52"/>
-      <c r="G71" s="46"/>
-      <c r="H71" s="61"/>
-      <c r="I71" s="61"/>
-      <c r="J71" s="46"/>
+      <c r="D71" s="80"/>
+      <c r="E71" s="83"/>
+      <c r="G71" s="77"/>
+      <c r="H71" s="89"/>
+      <c r="I71" s="89"/>
+      <c r="J71" s="77"/>
       <c r="L71" s="55"/>
-      <c r="M71" s="58"/>
-      <c r="N71" s="58"/>
+      <c r="M71" s="86"/>
+      <c r="N71" s="86"/>
       <c r="O71" s="55"/>
-      <c r="Q71" s="64"/>
-      <c r="R71" s="64"/>
-      <c r="S71" s="64"/>
+      <c r="Q71" s="92"/>
+      <c r="R71" s="92"/>
+      <c r="S71" s="92"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D72" s="49"/>
-      <c r="E72" s="52"/>
-      <c r="G72" s="46"/>
-      <c r="H72" s="61"/>
-      <c r="I72" s="61"/>
-      <c r="J72" s="46"/>
+      <c r="D72" s="80"/>
+      <c r="E72" s="83"/>
+      <c r="G72" s="77"/>
+      <c r="H72" s="89"/>
+      <c r="I72" s="89"/>
+      <c r="J72" s="77"/>
       <c r="L72" s="55"/>
-      <c r="M72" s="58"/>
-      <c r="N72" s="58"/>
+      <c r="M72" s="86"/>
+      <c r="N72" s="86"/>
       <c r="O72" s="55"/>
-      <c r="Q72" s="64"/>
-      <c r="R72" s="64"/>
-      <c r="S72" s="64"/>
+      <c r="Q72" s="92"/>
+      <c r="R72" s="92"/>
+      <c r="S72" s="92"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D73" s="49"/>
-      <c r="E73" s="52"/>
-      <c r="G73" s="46"/>
-      <c r="H73" s="61"/>
-      <c r="I73" s="61"/>
-      <c r="J73" s="46"/>
+      <c r="D73" s="80"/>
+      <c r="E73" s="83"/>
+      <c r="G73" s="77"/>
+      <c r="H73" s="89"/>
+      <c r="I73" s="89"/>
+      <c r="J73" s="77"/>
       <c r="L73" s="55"/>
-      <c r="M73" s="58"/>
-      <c r="N73" s="58"/>
+      <c r="M73" s="86"/>
+      <c r="N73" s="86"/>
       <c r="O73" s="55"/>
-      <c r="Q73" s="64"/>
-      <c r="R73" s="64"/>
-      <c r="S73" s="64"/>
+      <c r="Q73" s="92"/>
+      <c r="R73" s="92"/>
+      <c r="S73" s="92"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D74" s="49"/>
-      <c r="E74" s="52"/>
-      <c r="G74" s="46"/>
-      <c r="H74" s="61"/>
-      <c r="I74" s="61"/>
-      <c r="J74" s="46"/>
+      <c r="D74" s="80"/>
+      <c r="E74" s="83"/>
+      <c r="G74" s="77"/>
+      <c r="H74" s="89"/>
+      <c r="I74" s="89"/>
+      <c r="J74" s="77"/>
       <c r="L74" s="55"/>
-      <c r="M74" s="58"/>
-      <c r="N74" s="58"/>
+      <c r="M74" s="86"/>
+      <c r="N74" s="86"/>
       <c r="O74" s="55"/>
-      <c r="Q74" s="64"/>
-      <c r="R74" s="64"/>
-      <c r="S74" s="64"/>
+      <c r="Q74" s="92"/>
+      <c r="R74" s="92"/>
+      <c r="S74" s="92"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D75" s="50"/>
-      <c r="E75" s="53"/>
-      <c r="G75" s="47"/>
-      <c r="H75" s="62"/>
-      <c r="I75" s="62"/>
-      <c r="J75" s="47"/>
+      <c r="D75" s="81"/>
+      <c r="E75" s="84"/>
+      <c r="G75" s="78"/>
+      <c r="H75" s="90"/>
+      <c r="I75" s="90"/>
+      <c r="J75" s="78"/>
       <c r="L75" s="56"/>
-      <c r="M75" s="59"/>
-      <c r="N75" s="59"/>
+      <c r="M75" s="87"/>
+      <c r="N75" s="87"/>
       <c r="O75" s="56"/>
-      <c r="Q75" s="65"/>
-      <c r="R75" s="65"/>
-      <c r="S75" s="65"/>
+      <c r="Q75" s="93"/>
+      <c r="R75" s="93"/>
+      <c r="S75" s="93"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -9191,6 +9192,15 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>